<commit_message>
release: finalize NKT Management System v1.0.1
</commit_message>
<xml_diff>
--- a/templates/BB_ong_hong.xlsx
+++ b/templates/BB_ong_hong.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\6. Report NKT XCO-TBDG\NKT Report_2026\NKT-Report\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC1E0215-4D2C-46FD-9C0E-05087B4384BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BC04A26-2124-4893-94C7-722AA772005A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="87">
   <si>
     <t>Xưởng Cần ống &amp; Thiết bị đầu giếng - Ban Thiết bị dầu khí - XNCĐ</t>
   </si>
@@ -310,15 +310,22 @@
   </si>
   <si>
     <t>71H6.26</t>
+  </si>
+  <si>
+    <t>2205/BK-22</t>
+  </si>
+  <si>
+    <t>HKT-SC-39/26</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.000000"/>
     <numFmt numFmtId="165" formatCode="0&quot;bar&quot;"/>
+    <numFmt numFmtId="166" formatCode="[$-409]d\-mmm\-yyyy;@"/>
   </numFmts>
   <fonts count="14" x14ac:knownFonts="1">
     <font>
@@ -409,7 +416,7 @@
       <family val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -425,6 +432,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF2CC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -554,7 +567,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2"/>
@@ -685,6 +698,8 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -824,7 +839,7 @@
       <xdr:col>4</xdr:col>
       <xdr:colOff>90741</xdr:colOff>
       <xdr:row>54</xdr:row>
-      <xdr:rowOff>59634</xdr:rowOff>
+      <xdr:rowOff>59635</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -873,7 +888,7 @@
       <xdr:col>12</xdr:col>
       <xdr:colOff>89154</xdr:colOff>
       <xdr:row>54</xdr:row>
-      <xdr:rowOff>6625</xdr:rowOff>
+      <xdr:rowOff>6626</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -971,7 +986,7 @@
       <xdr:col>3</xdr:col>
       <xdr:colOff>1475</xdr:colOff>
       <xdr:row>54</xdr:row>
-      <xdr:rowOff>54997</xdr:rowOff>
+      <xdr:rowOff>54998</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1159,7 +1174,7 @@
       <xdr:col>7</xdr:col>
       <xdr:colOff>4093</xdr:colOff>
       <xdr:row>54</xdr:row>
-      <xdr:rowOff>79730</xdr:rowOff>
+      <xdr:rowOff>79731</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1850,42 +1865,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:34" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="52" t="s">
+      <c r="A1" s="54" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="53"/>
-      <c r="C1" s="53"/>
-      <c r="D1" s="53"/>
-      <c r="E1" s="53"/>
-      <c r="F1" s="53"/>
-      <c r="G1" s="53"/>
-      <c r="H1" s="53"/>
-      <c r="I1" s="53"/>
+      <c r="B1" s="55"/>
+      <c r="C1" s="55"/>
+      <c r="D1" s="55"/>
+      <c r="E1" s="55"/>
+      <c r="F1" s="55"/>
+      <c r="G1" s="55"/>
+      <c r="H1" s="55"/>
+      <c r="I1" s="55"/>
       <c r="J1" s="34"/>
       <c r="K1" s="34"/>
-      <c r="L1" s="65" t="s">
+      <c r="L1" s="67" t="s">
         <v>1</v>
       </c>
-      <c r="M1" s="53"/>
-      <c r="N1" s="53"/>
+      <c r="M1" s="55"/>
+      <c r="N1" s="55"/>
     </row>
     <row r="2" spans="1:34" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="66" t="s">
+      <c r="A2" s="68" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="53"/>
-      <c r="C2" s="53"/>
-      <c r="D2" s="53"/>
-      <c r="E2" s="53"/>
-      <c r="F2" s="53"/>
-      <c r="G2" s="53"/>
-      <c r="H2" s="53"/>
-      <c r="I2" s="53"/>
-      <c r="J2" s="53"/>
-      <c r="K2" s="53"/>
-      <c r="L2" s="53"/>
-      <c r="M2" s="53"/>
-      <c r="N2" s="53"/>
+      <c r="B2" s="55"/>
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
+      <c r="H2" s="55"/>
+      <c r="I2" s="55"/>
+      <c r="J2" s="55"/>
+      <c r="K2" s="55"/>
+      <c r="L2" s="55"/>
+      <c r="M2" s="55"/>
+      <c r="N2" s="55"/>
     </row>
     <row r="3" spans="1:34" s="1" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="35"/>
@@ -1949,7 +1964,9 @@
         <v>11</v>
       </c>
       <c r="G6" s="43"/>
-      <c r="I6" s="43"/>
+      <c r="I6" s="52" t="s">
+        <v>85</v>
+      </c>
       <c r="K6" s="34"/>
     </row>
     <row r="7" spans="1:34" s="39" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1966,12 +1983,16 @@
         <v>13</v>
       </c>
       <c r="G7" s="43"/>
-      <c r="I7" s="43"/>
+      <c r="I7" s="52" t="s">
+        <v>86</v>
+      </c>
       <c r="L7" s="34"/>
       <c r="M7" s="40" t="s">
         <v>14</v>
       </c>
-      <c r="N7" s="43"/>
+      <c r="N7" s="53">
+        <v>46199</v>
+      </c>
     </row>
     <row r="8" spans="1:34" s="39" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="36" t="s">
@@ -1995,75 +2016,75 @@
       <c r="N8" s="34"/>
     </row>
     <row r="9" spans="1:34" s="39" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="72" t="s">
+      <c r="A9" s="74" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="59"/>
-      <c r="C9" s="59"/>
-      <c r="D9" s="58" t="s">
+      <c r="B9" s="61"/>
+      <c r="C9" s="61"/>
+      <c r="D9" s="60" t="s">
         <v>84</v>
       </c>
-      <c r="E9" s="59"/>
-      <c r="F9" s="73" t="s">
+      <c r="E9" s="61"/>
+      <c r="F9" s="75" t="s">
         <v>20</v>
       </c>
-      <c r="G9" s="59"/>
-      <c r="H9" s="59"/>
-      <c r="I9" s="59"/>
-      <c r="J9" s="59"/>
-      <c r="K9" s="59"/>
-      <c r="L9" s="59"/>
-      <c r="M9" s="59"/>
+      <c r="G9" s="61"/>
+      <c r="H9" s="61"/>
+      <c r="I9" s="61"/>
+      <c r="J9" s="61"/>
+      <c r="K9" s="61"/>
+      <c r="L9" s="61"/>
+      <c r="M9" s="61"/>
       <c r="N9" s="46"/>
     </row>
     <row r="10" spans="1:34" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="60" t="s">
+      <c r="A10" s="62" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="74" t="s">
+      <c r="B10" s="76" t="s">
         <v>22</v>
       </c>
-      <c r="C10" s="60" t="s">
+      <c r="C10" s="62" t="s">
         <v>23</v>
       </c>
-      <c r="D10" s="75" t="s">
+      <c r="D10" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="E10" s="60" t="s">
+      <c r="E10" s="62" t="s">
         <v>25</v>
       </c>
-      <c r="F10" s="60" t="s">
+      <c r="F10" s="62" t="s">
         <v>26</v>
       </c>
-      <c r="G10" s="60" t="s">
+      <c r="G10" s="62" t="s">
         <v>27</v>
       </c>
-      <c r="H10" s="60" t="s">
+      <c r="H10" s="62" t="s">
         <v>28</v>
       </c>
-      <c r="I10" s="62"/>
-      <c r="J10" s="71" t="s">
+      <c r="I10" s="64"/>
+      <c r="J10" s="73" t="s">
         <v>29</v>
       </c>
-      <c r="K10" s="62"/>
-      <c r="L10" s="60" t="s">
+      <c r="K10" s="64"/>
+      <c r="L10" s="62" t="s">
         <v>30</v>
       </c>
-      <c r="M10" s="60" t="s">
+      <c r="M10" s="62" t="s">
         <v>31</v>
       </c>
-      <c r="N10" s="70" t="s">
+      <c r="N10" s="72" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:34" s="1" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="61"/>
-      <c r="B11" s="61"/>
-      <c r="C11" s="61"/>
-      <c r="D11" s="61"/>
-      <c r="E11" s="61"/>
-      <c r="F11" s="61"/>
-      <c r="G11" s="61"/>
+      <c r="A11" s="63"/>
+      <c r="B11" s="63"/>
+      <c r="C11" s="63"/>
+      <c r="D11" s="63"/>
+      <c r="E11" s="63"/>
+      <c r="F11" s="63"/>
+      <c r="G11" s="63"/>
       <c r="H11" s="48" t="s">
         <v>33</v>
       </c>
@@ -2076,15 +2097,15 @@
       <c r="K11" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="L11" s="61"/>
-      <c r="M11" s="61"/>
-      <c r="N11" s="61"/>
+      <c r="L11" s="63"/>
+      <c r="M11" s="63"/>
+      <c r="N11" s="63"/>
     </row>
     <row r="12" spans="1:34" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="60" t="s">
+      <c r="A12" s="62" t="s">
         <v>37</v>
       </c>
-      <c r="B12" s="62"/>
+      <c r="B12" s="64"/>
       <c r="C12" s="20"/>
       <c r="D12" s="8">
         <v>8.4437499999999996</v>
@@ -2094,10 +2115,10 @@
       </c>
       <c r="F12" s="20"/>
       <c r="G12" s="20"/>
-      <c r="H12" s="60" t="s">
+      <c r="H12" s="62" t="s">
         <v>39</v>
       </c>
-      <c r="I12" s="62"/>
+      <c r="I12" s="64"/>
       <c r="J12" s="20"/>
       <c r="K12" s="20"/>
       <c r="L12" s="49" t="s">
@@ -2119,7 +2140,7 @@
       <c r="C13" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="D13" s="63" t="s">
+      <c r="D13" s="65" t="s">
         <v>61</v>
       </c>
       <c r="E13" s="6" t="s">
@@ -2167,7 +2188,7 @@
       <c r="C14" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="D14" s="64"/>
+      <c r="D14" s="66"/>
       <c r="E14" s="6" t="s">
         <v>41</v>
       </c>
@@ -2213,7 +2234,7 @@
       <c r="C15" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="D15" s="64"/>
+      <c r="D15" s="66"/>
       <c r="E15" s="6" t="s">
         <v>41</v>
       </c>
@@ -2259,7 +2280,7 @@
       <c r="C16" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="D16" s="64"/>
+      <c r="D16" s="66"/>
       <c r="E16" s="6" t="s">
         <v>41</v>
       </c>
@@ -2305,7 +2326,7 @@
       <c r="C17" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="D17" s="64"/>
+      <c r="D17" s="66"/>
       <c r="E17" s="6" t="s">
         <v>41</v>
       </c>
@@ -2348,7 +2369,7 @@
       <c r="C18" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="D18" s="64"/>
+      <c r="D18" s="66"/>
       <c r="E18" s="6" t="s">
         <v>41</v>
       </c>
@@ -2391,7 +2412,7 @@
       <c r="C19" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="D19" s="64"/>
+      <c r="D19" s="66"/>
       <c r="E19" s="6" t="s">
         <v>41</v>
       </c>
@@ -2434,7 +2455,7 @@
       <c r="C20" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="D20" s="64"/>
+      <c r="D20" s="66"/>
       <c r="E20" s="6" t="s">
         <v>41</v>
       </c>
@@ -2477,7 +2498,7 @@
       <c r="C21" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="D21" s="64"/>
+      <c r="D21" s="66"/>
       <c r="E21" s="6" t="s">
         <v>41</v>
       </c>
@@ -2520,7 +2541,7 @@
       <c r="C22" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="D22" s="64"/>
+      <c r="D22" s="66"/>
       <c r="E22" s="6" t="s">
         <v>41</v>
       </c>
@@ -2563,7 +2584,7 @@
       <c r="C23" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="D23" s="64"/>
+      <c r="D23" s="66"/>
       <c r="E23" s="6" t="s">
         <v>41</v>
       </c>
@@ -2606,7 +2627,7 @@
       <c r="C24" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="D24" s="64"/>
+      <c r="D24" s="66"/>
       <c r="E24" s="6" t="s">
         <v>41</v>
       </c>
@@ -2649,7 +2670,7 @@
       <c r="C25" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="D25" s="64"/>
+      <c r="D25" s="66"/>
       <c r="E25" s="6" t="s">
         <v>41</v>
       </c>
@@ -2692,7 +2713,7 @@
       <c r="C26" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="D26" s="64"/>
+      <c r="D26" s="66"/>
       <c r="E26" s="6" t="s">
         <v>41</v>
       </c>
@@ -2735,7 +2756,7 @@
       <c r="C27" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="D27" s="64"/>
+      <c r="D27" s="66"/>
       <c r="E27" s="6" t="s">
         <v>41</v>
       </c>
@@ -2768,13 +2789,13 @@
       </c>
       <c r="O27" s="11"/>
     </row>
-    <row r="28" spans="1:15" s="1" customFormat="1" ht="14.65" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:15" s="1" customFormat="1" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="6">
         <v>16</v>
       </c>
       <c r="B28" s="7"/>
       <c r="C28" s="6"/>
-      <c r="D28" s="64"/>
+      <c r="D28" s="66"/>
       <c r="E28" s="6"/>
       <c r="F28" s="9"/>
       <c r="G28" s="10"/>
@@ -2787,13 +2808,13 @@
       <c r="N28" s="51"/>
       <c r="O28" s="11"/>
     </row>
-    <row r="29" spans="1:15" s="1" customFormat="1" ht="14.65" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:15" s="1" customFormat="1" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="6">
         <v>17</v>
       </c>
       <c r="B29" s="7"/>
       <c r="C29" s="6"/>
-      <c r="D29" s="64"/>
+      <c r="D29" s="66"/>
       <c r="E29" s="6"/>
       <c r="F29" s="9"/>
       <c r="G29" s="10"/>
@@ -2806,13 +2827,13 @@
       <c r="N29" s="51"/>
       <c r="O29" s="11"/>
     </row>
-    <row r="30" spans="1:15" s="1" customFormat="1" ht="14.65" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:15" s="1" customFormat="1" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="6">
         <v>18</v>
       </c>
       <c r="B30" s="7"/>
       <c r="C30" s="6"/>
-      <c r="D30" s="64"/>
+      <c r="D30" s="66"/>
       <c r="E30" s="6"/>
       <c r="F30" s="9"/>
       <c r="G30" s="10"/>
@@ -2825,13 +2846,13 @@
       <c r="N30" s="51"/>
       <c r="O30" s="11"/>
     </row>
-    <row r="31" spans="1:15" s="1" customFormat="1" ht="14.65" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:15" s="1" customFormat="1" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="6">
         <v>19</v>
       </c>
       <c r="B31" s="7"/>
       <c r="C31" s="6"/>
-      <c r="D31" s="64"/>
+      <c r="D31" s="66"/>
       <c r="E31" s="6"/>
       <c r="F31" s="9"/>
       <c r="G31" s="10"/>
@@ -2844,13 +2865,13 @@
       <c r="N31" s="51"/>
       <c r="O31" s="11"/>
     </row>
-    <row r="32" spans="1:15" s="1" customFormat="1" ht="14.65" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:15" s="1" customFormat="1" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="6">
         <v>20</v>
       </c>
       <c r="B32" s="7"/>
       <c r="C32" s="6"/>
-      <c r="D32" s="64"/>
+      <c r="D32" s="66"/>
       <c r="E32" s="6"/>
       <c r="F32" s="9"/>
       <c r="G32" s="10"/>
@@ -2863,13 +2884,13 @@
       <c r="N32" s="51"/>
       <c r="O32" s="11"/>
     </row>
-    <row r="33" spans="1:34" s="1" customFormat="1" ht="14.65" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:34" s="1" customFormat="1" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="6">
         <v>21</v>
       </c>
       <c r="B33" s="7"/>
       <c r="C33" s="6"/>
-      <c r="D33" s="64"/>
+      <c r="D33" s="66"/>
       <c r="E33" s="6"/>
       <c r="F33" s="9"/>
       <c r="G33" s="10"/>
@@ -2882,13 +2903,13 @@
       <c r="N33" s="51"/>
       <c r="O33" s="11"/>
     </row>
-    <row r="34" spans="1:34" s="1" customFormat="1" ht="14.65" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:34" s="1" customFormat="1" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="6">
         <v>22</v>
       </c>
       <c r="B34" s="7"/>
       <c r="C34" s="6"/>
-      <c r="D34" s="64"/>
+      <c r="D34" s="66"/>
       <c r="E34" s="6"/>
       <c r="F34" s="9"/>
       <c r="G34" s="10"/>
@@ -2901,13 +2922,13 @@
       <c r="N34" s="51"/>
       <c r="O34" s="11"/>
     </row>
-    <row r="35" spans="1:34" s="1" customFormat="1" ht="14.65" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:34" s="1" customFormat="1" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="6">
         <v>23</v>
       </c>
       <c r="B35" s="7"/>
       <c r="C35" s="6"/>
-      <c r="D35" s="64"/>
+      <c r="D35" s="66"/>
       <c r="E35" s="6"/>
       <c r="F35" s="9"/>
       <c r="G35" s="10"/>
@@ -2920,13 +2941,13 @@
       <c r="N35" s="51"/>
       <c r="O35" s="11"/>
     </row>
-    <row r="36" spans="1:34" s="1" customFormat="1" ht="14.65" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:34" s="1" customFormat="1" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="6">
         <v>24</v>
       </c>
       <c r="B36" s="7"/>
       <c r="C36" s="6"/>
-      <c r="D36" s="64"/>
+      <c r="D36" s="66"/>
       <c r="E36" s="6"/>
       <c r="F36" s="9"/>
       <c r="G36" s="10"/>
@@ -2939,13 +2960,13 @@
       <c r="N36" s="51"/>
       <c r="O36" s="11"/>
     </row>
-    <row r="37" spans="1:34" s="1" customFormat="1" ht="14.65" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:34" s="1" customFormat="1" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="6">
         <v>25</v>
       </c>
       <c r="B37" s="7"/>
       <c r="C37" s="6"/>
-      <c r="D37" s="64"/>
+      <c r="D37" s="66"/>
       <c r="E37" s="6"/>
       <c r="F37" s="9"/>
       <c r="G37" s="10"/>
@@ -2958,13 +2979,13 @@
       <c r="N37" s="51"/>
       <c r="O37" s="11"/>
     </row>
-    <row r="38" spans="1:34" s="1" customFormat="1" ht="14.65" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:34" s="1" customFormat="1" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="6">
         <v>26</v>
       </c>
       <c r="B38" s="7"/>
       <c r="C38" s="6"/>
-      <c r="D38" s="64"/>
+      <c r="D38" s="66"/>
       <c r="E38" s="6"/>
       <c r="F38" s="9"/>
       <c r="G38" s="10"/>
@@ -2977,13 +2998,13 @@
       <c r="N38" s="51"/>
       <c r="O38" s="11"/>
     </row>
-    <row r="39" spans="1:34" s="1" customFormat="1" ht="14.65" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:34" s="1" customFormat="1" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="6">
         <v>27</v>
       </c>
       <c r="B39" s="7"/>
       <c r="C39" s="6"/>
-      <c r="D39" s="64"/>
+      <c r="D39" s="66"/>
       <c r="E39" s="6"/>
       <c r="F39" s="9"/>
       <c r="G39" s="10"/>
@@ -2996,13 +3017,13 @@
       <c r="N39" s="51"/>
       <c r="O39" s="11"/>
     </row>
-    <row r="40" spans="1:34" s="1" customFormat="1" ht="14.65" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:34" s="1" customFormat="1" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="6">
         <v>28</v>
       </c>
       <c r="B40" s="7"/>
       <c r="C40" s="6"/>
-      <c r="D40" s="64"/>
+      <c r="D40" s="66"/>
       <c r="E40" s="6"/>
       <c r="F40" s="9"/>
       <c r="G40" s="10"/>
@@ -3015,13 +3036,13 @@
       <c r="N40" s="51"/>
       <c r="O40" s="11"/>
     </row>
-    <row r="41" spans="1:34" s="1" customFormat="1" ht="14.65" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:34" s="1" customFormat="1" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="6">
         <v>29</v>
       </c>
       <c r="B41" s="7"/>
       <c r="C41" s="6"/>
-      <c r="D41" s="64"/>
+      <c r="D41" s="66"/>
       <c r="E41" s="6"/>
       <c r="F41" s="9"/>
       <c r="G41" s="10"/>
@@ -3034,13 +3055,13 @@
       <c r="N41" s="51"/>
       <c r="O41" s="11"/>
     </row>
-    <row r="42" spans="1:34" s="1" customFormat="1" ht="14.65" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:34" s="1" customFormat="1" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="6">
         <v>30</v>
       </c>
       <c r="B42" s="7"/>
       <c r="C42" s="6"/>
-      <c r="D42" s="64"/>
+      <c r="D42" s="66"/>
       <c r="E42" s="6"/>
       <c r="F42" s="9"/>
       <c r="G42" s="10"/>
@@ -3053,13 +3074,13 @@
       <c r="N42" s="51"/>
       <c r="O42" s="11"/>
     </row>
-    <row r="43" spans="1:34" s="1" customFormat="1" ht="14.65" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:34" s="1" customFormat="1" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="6">
         <v>31</v>
       </c>
       <c r="B43" s="7"/>
       <c r="C43" s="6"/>
-      <c r="D43" s="64"/>
+      <c r="D43" s="66"/>
       <c r="E43" s="6"/>
       <c r="F43" s="9"/>
       <c r="G43" s="10"/>
@@ -3072,13 +3093,13 @@
       <c r="N43" s="51"/>
       <c r="O43" s="11"/>
     </row>
-    <row r="44" spans="1:34" s="1" customFormat="1" ht="14.65" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:34" s="1" customFormat="1" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="6">
         <v>32</v>
       </c>
       <c r="B44" s="7"/>
       <c r="C44" s="6"/>
-      <c r="D44" s="64"/>
+      <c r="D44" s="66"/>
       <c r="E44" s="6"/>
       <c r="F44" s="9"/>
       <c r="G44" s="10"/>
@@ -3091,13 +3112,13 @@
       <c r="N44" s="51"/>
       <c r="O44" s="11"/>
     </row>
-    <row r="45" spans="1:34" s="1" customFormat="1" ht="14.65" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:34" s="1" customFormat="1" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="6">
         <v>33</v>
       </c>
       <c r="B45" s="7"/>
       <c r="C45" s="6"/>
-      <c r="D45" s="64"/>
+      <c r="D45" s="66"/>
       <c r="E45" s="6"/>
       <c r="F45" s="9"/>
       <c r="G45" s="10"/>
@@ -3113,13 +3134,13 @@
         <v>19</v>
       </c>
     </row>
-    <row r="46" spans="1:34" s="1" customFormat="1" ht="14.65" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:34" s="1" customFormat="1" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="6">
         <v>34</v>
       </c>
       <c r="B46" s="7"/>
       <c r="C46" s="6"/>
-      <c r="D46" s="64"/>
+      <c r="D46" s="66"/>
       <c r="E46" s="6"/>
       <c r="F46" s="9"/>
       <c r="G46" s="10"/>
@@ -3132,13 +3153,13 @@
       <c r="N46" s="51"/>
       <c r="O46" s="11"/>
     </row>
-    <row r="47" spans="1:34" s="1" customFormat="1" ht="14.65" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:34" s="1" customFormat="1" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="6">
         <v>35</v>
       </c>
       <c r="B47" s="7"/>
       <c r="C47" s="6"/>
-      <c r="D47" s="64"/>
+      <c r="D47" s="66"/>
       <c r="E47" s="6"/>
       <c r="F47" s="9"/>
       <c r="G47" s="10"/>
@@ -3151,13 +3172,13 @@
       <c r="N47" s="51"/>
       <c r="O47" s="11"/>
     </row>
-    <row r="48" spans="1:34" s="1" customFormat="1" ht="14.65" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:34" s="1" customFormat="1" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="6">
         <v>36</v>
       </c>
       <c r="B48" s="7"/>
       <c r="C48" s="6"/>
-      <c r="D48" s="64"/>
+      <c r="D48" s="66"/>
       <c r="E48" s="6"/>
       <c r="F48" s="9"/>
       <c r="G48" s="10"/>
@@ -3170,13 +3191,13 @@
       <c r="N48" s="51"/>
       <c r="O48" s="11"/>
     </row>
-    <row r="49" spans="1:43" s="1" customFormat="1" ht="14.65" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:43" s="1" customFormat="1" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="6">
         <v>37</v>
       </c>
       <c r="B49" s="7"/>
       <c r="C49" s="6"/>
-      <c r="D49" s="64"/>
+      <c r="D49" s="66"/>
       <c r="E49" s="6"/>
       <c r="F49" s="9"/>
       <c r="G49" s="10"/>
@@ -3189,13 +3210,13 @@
       <c r="N49" s="51"/>
       <c r="O49" s="11"/>
     </row>
-    <row r="50" spans="1:43" s="1" customFormat="1" ht="14.65" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:43" s="1" customFormat="1" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="6">
         <v>38</v>
       </c>
       <c r="B50" s="7"/>
       <c r="C50" s="6"/>
-      <c r="D50" s="64"/>
+      <c r="D50" s="66"/>
       <c r="E50" s="6"/>
       <c r="F50" s="9"/>
       <c r="G50" s="10"/>
@@ -3208,13 +3229,13 @@
       <c r="N50" s="51"/>
       <c r="O50" s="11"/>
     </row>
-    <row r="51" spans="1:43" s="1" customFormat="1" ht="14.65" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:43" s="1" customFormat="1" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="6">
         <v>39</v>
       </c>
       <c r="B51" s="7"/>
       <c r="C51" s="6"/>
-      <c r="D51" s="64"/>
+      <c r="D51" s="66"/>
       <c r="E51" s="6"/>
       <c r="F51" s="9"/>
       <c r="G51" s="10"/>
@@ -3227,13 +3248,13 @@
       <c r="N51" s="51"/>
       <c r="O51" s="11"/>
     </row>
-    <row r="52" spans="1:43" s="1" customFormat="1" ht="14.65" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:43" s="1" customFormat="1" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="6">
         <v>40</v>
       </c>
       <c r="B52" s="7"/>
       <c r="C52" s="6"/>
-      <c r="D52" s="64"/>
+      <c r="D52" s="66"/>
       <c r="E52" s="6"/>
       <c r="F52" s="9"/>
       <c r="G52" s="10"/>
@@ -3247,10 +3268,10 @@
       <c r="O52" s="11"/>
     </row>
     <row r="53" spans="1:43" s="1" customFormat="1" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="60" t="s">
+      <c r="A53" s="62" t="s">
         <v>44</v>
       </c>
-      <c r="B53" s="62"/>
+      <c r="B53" s="64"/>
       <c r="C53" s="21" t="s">
         <v>45</v>
       </c>
@@ -3287,10 +3308,10 @@
       <c r="N53" s="24"/>
     </row>
     <row r="54" spans="1:43" s="1" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="60" t="s">
+      <c r="A54" s="62" t="s">
         <v>52</v>
       </c>
-      <c r="B54" s="62"/>
+      <c r="B54" s="64"/>
       <c r="C54" s="25"/>
       <c r="D54" s="26"/>
       <c r="E54" s="21"/>
@@ -3305,19 +3326,19 @@
       <c r="N54" s="28"/>
     </row>
     <row r="55" spans="1:43" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B55" s="68" t="s">
+      <c r="B55" s="70" t="s">
         <v>53</v>
       </c>
-      <c r="C55" s="69"/>
-      <c r="D55" s="69"/>
-      <c r="E55" s="69"/>
-      <c r="F55" s="69"/>
-      <c r="G55" s="69"/>
-      <c r="H55" s="69"/>
-      <c r="I55" s="69"/>
-      <c r="J55" s="69"/>
-      <c r="K55" s="69"/>
-      <c r="L55" s="69"/>
+      <c r="C55" s="71"/>
+      <c r="D55" s="71"/>
+      <c r="E55" s="71"/>
+      <c r="F55" s="71"/>
+      <c r="G55" s="71"/>
+      <c r="H55" s="71"/>
+      <c r="I55" s="71"/>
+      <c r="J55" s="71"/>
+      <c r="K55" s="71"/>
+      <c r="L55" s="71"/>
       <c r="M55" s="29"/>
       <c r="N55" s="29"/>
     </row>
@@ -3362,34 +3383,34 @@
       </c>
     </row>
     <row r="58" spans="1:43" s="13" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="67" t="s">
+      <c r="A58" s="69" t="s">
         <v>57</v>
       </c>
-      <c r="B58" s="55"/>
-      <c r="C58" s="55"/>
-      <c r="D58" s="55"/>
-      <c r="E58" s="55"/>
-      <c r="F58" s="55"/>
-      <c r="G58" s="55"/>
-      <c r="H58" s="55"/>
-      <c r="I58" s="55"/>
-      <c r="J58" s="55"/>
-      <c r="K58" s="55"/>
-      <c r="L58" s="55"/>
-      <c r="M58" s="55"/>
-      <c r="N58" s="55"/>
-      <c r="Q58" s="56"/>
-      <c r="R58" s="55"/>
-      <c r="S58" s="55"/>
-      <c r="T58" s="54"/>
-      <c r="U58" s="55"/>
-      <c r="V58" s="55"/>
-      <c r="W58" s="57"/>
-      <c r="X58" s="55"/>
-      <c r="Y58" s="55"/>
-      <c r="Z58" s="57"/>
-      <c r="AA58" s="55"/>
-      <c r="AB58" s="55"/>
+      <c r="B58" s="57"/>
+      <c r="C58" s="57"/>
+      <c r="D58" s="57"/>
+      <c r="E58" s="57"/>
+      <c r="F58" s="57"/>
+      <c r="G58" s="57"/>
+      <c r="H58" s="57"/>
+      <c r="I58" s="57"/>
+      <c r="J58" s="57"/>
+      <c r="K58" s="57"/>
+      <c r="L58" s="57"/>
+      <c r="M58" s="57"/>
+      <c r="N58" s="57"/>
+      <c r="Q58" s="58"/>
+      <c r="R58" s="57"/>
+      <c r="S58" s="57"/>
+      <c r="T58" s="56"/>
+      <c r="U58" s="57"/>
+      <c r="V58" s="57"/>
+      <c r="W58" s="59"/>
+      <c r="X58" s="57"/>
+      <c r="Y58" s="57"/>
+      <c r="Z58" s="59"/>
+      <c r="AA58" s="57"/>
+      <c r="AB58" s="57"/>
     </row>
     <row r="59" spans="1:43" s="13" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="17"/>
@@ -3440,34 +3461,34 @@
       <c r="N61" s="19"/>
     </row>
     <row r="62" spans="1:43" s="13" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="67" t="s">
+      <c r="A62" s="69" t="s">
         <v>58</v>
       </c>
-      <c r="B62" s="55"/>
-      <c r="C62" s="55"/>
-      <c r="D62" s="55"/>
-      <c r="E62" s="55"/>
-      <c r="F62" s="55"/>
-      <c r="G62" s="55"/>
-      <c r="H62" s="55"/>
-      <c r="I62" s="55"/>
-      <c r="J62" s="55"/>
-      <c r="K62" s="55"/>
-      <c r="L62" s="55"/>
-      <c r="M62" s="55"/>
-      <c r="N62" s="55"/>
-      <c r="Q62" s="56"/>
-      <c r="R62" s="55"/>
-      <c r="S62" s="55"/>
-      <c r="T62" s="54"/>
-      <c r="U62" s="55"/>
-      <c r="V62" s="55"/>
-      <c r="W62" s="57"/>
-      <c r="X62" s="55"/>
-      <c r="Y62" s="55"/>
-      <c r="Z62" s="57"/>
-      <c r="AA62" s="55"/>
-      <c r="AB62" s="55"/>
+      <c r="B62" s="57"/>
+      <c r="C62" s="57"/>
+      <c r="D62" s="57"/>
+      <c r="E62" s="57"/>
+      <c r="F62" s="57"/>
+      <c r="G62" s="57"/>
+      <c r="H62" s="57"/>
+      <c r="I62" s="57"/>
+      <c r="J62" s="57"/>
+      <c r="K62" s="57"/>
+      <c r="L62" s="57"/>
+      <c r="M62" s="57"/>
+      <c r="N62" s="57"/>
+      <c r="Q62" s="58"/>
+      <c r="R62" s="57"/>
+      <c r="S62" s="57"/>
+      <c r="T62" s="56"/>
+      <c r="U62" s="57"/>
+      <c r="V62" s="57"/>
+      <c r="W62" s="59"/>
+      <c r="X62" s="57"/>
+      <c r="Y62" s="57"/>
+      <c r="Z62" s="59"/>
+      <c r="AA62" s="57"/>
+      <c r="AB62" s="57"/>
     </row>
   </sheetData>
   <mergeCells count="34">

</xml_diff>